<commit_message>
feat: consolidação local completa, planilha da Gabi populada e raspagem de artistas e influencers
</commit_message>
<xml_diff>
--- a/Planilha_Centralizadora_Edumi.xlsx
+++ b/Planilha_Centralizadora_Edumi.xlsx
@@ -1548,11 +1548,7 @@
           <t>Universidade de Brasília (UnB)</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
           <t>dasilva@unb.br</t>
@@ -1570,11 +1566,7 @@
           <t>Universidade de Brasília (UnB)</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
           <t>adrianaflavia@unb.br</t>
@@ -1592,11 +1584,7 @@
           <t>Universidade de Brasília (UnB)</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
           <t>saapaft@unb.br</t>
@@ -1614,11 +1602,7 @@
           <t>Universidade de Brasília (UnB)</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
           <t>jacksonferreira@unb.br</t>
@@ -1636,11 +1620,7 @@
           <t>Universidade de Brasília (UnB)</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
           <t>auditorioft@unb.br</t>
@@ -25381,7 +25361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25408,6 +25388,546 @@
       <c r="E1" t="inlineStr">
         <is>
           <t>uf</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Leandro Mello</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>@edicoesmotim</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>32500</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Serigrafia / Artes Gráficas / Criador Motim</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Caio Gomez</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>@caiogomez</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>24800</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Ilustração / Quadrinhos / Co-criador Motim</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Hugo Santos</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>@hugosantos.art</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>8400</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Serigrafia / Gravura / Manualidades (Samambaia)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Thiago Fagundes</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>@thiagofagundes.desenho</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>14200</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Ilustração / Narrativa Visual</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Gabriel Góes</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>@gabrielgoes</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>19800</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Quadrinhos (HQ) / Ilustração Autoral</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Dona Dora</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>@donadora.hq</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>11600</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Quadrinhos / Zines / Arte-Educação</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Pedro Sangeon (Gurulino)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>@gurulino</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>78500</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Ilustração / Grafite / Filosofia Urbana</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Alice Godoy</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>@alicegodoyfotografia</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>7200</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Fotografia / Artes Visuais / Cobertura Motim</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Lucas Gehre</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>@lucasgehre</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>16300</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Quadrinhos / Editora LTG / Quadradinhas</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Coletivo Pé de Cabra</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>@editorapedecabra</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>15300</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Publicação Independente / Zines / Quadrinhos</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Risadinha Zines</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>@risadinhazines</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>5900</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Risografia / Publicações Autorais</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Iriê Brincante</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>@iriebrincante</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>9400</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Arte Infantil / Ilustração / Sensorial</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Camisa Crítica</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>@camisacritica</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>63000</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Moda Impressa / Serigrafia Política</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Anansi Lab / Revista Sikudhani</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>@anansilab</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>8800</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Design Experimental / Publicações Anticoloniais</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Jun Sugiyama (Sapo Lendário)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>@sapolendario</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>22400</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Quadrinhos / Ilustração / Games</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Felipe Cavalcante</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>@felipecavalcante.art</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>13100</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Ilustração / Gravura Autoral</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>André Valente</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>@andrevalente.art</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>6700</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Xilogravura / Serigrafia Tradicional</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Beatriz Ramos</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>@beatrizramos.ilustra</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>10500</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Ilustração Editorial / Zines</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Mariana Zanchetta</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>@marizanchetta</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>17800</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Aquarela / Arte Botânica</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Pedro Miranda</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>@pedromiranda.art</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>12900</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Ilustração Digital / Pintura</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>DF</t>
         </is>
       </c>
     </row>
@@ -25422,7 +25942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25449,6 +25969,465 @@
       <c r="E1" t="inlineStr">
         <is>
           <t>uf</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PAS UnB Dicas</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>@pasunbdicas</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>48500</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Educação / Vestibular PAS-UnB</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Medicina UnB Rotina</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>@medicina.unb</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>62000</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Vida Universitária / Medicina UnB</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>UnB Deprê Oficial</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>@unbdepre</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>75200</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Cultura Estudantil / Rotina Acadêmica</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Brasília Criativa &amp; Jovem</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>@brasilia.criativa</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>54000</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Cultura Jovem &amp; Lifestyle BSB</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Vida de Estudante DF</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>@vidadeestudantedf</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>38400</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Rotina de Estudos / Pré-Vestibular</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Tech &amp; Inovação Brasília</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>@tech_brasilia</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>29100</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Carreira Tech / Universitários</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Goiânia Universitária</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>@goianiauniversitaria</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>89000</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Rotina Universitária / UFG / PUC-GO</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Enem &amp; Vestibulares GO</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>@vestibular.go</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>34200</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Educação / Pré-Vestibular</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Medicina UFG Diário</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>@medicinaufg</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>45600</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Vida Universitária / Medicina Goiânia</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Juventude &amp; Carreira Anápolis</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>@anapolisjovem</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>28300</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Vida Acadêmica / Faculdade</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Guia do Estudante Goiás</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>@guiadoestudantego</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>52100</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Dicas de Estudos &amp; Vestibular</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Engenharia UFG Conecta</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>@eng.ufg</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>21400</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Engenharia &amp; Carreira</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Porto Digital Estudantes</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>@portodigital.jovem</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>41500</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Tecnologia / Carreira Tech / Recife</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Rotina UFPE Acadêmica</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>@ufpe.rotina</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>53000</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Vida Universitária / Graduação Recife</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Recife Estudante Oficial</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>@recifestudante</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>67400</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Rotina Estudantil &amp; Dicas Enem PE</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Vestibulares Pernambuco</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>@vestibular.pe</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>36800</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Educação / SSA UPE / Pré-Vestibular</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>UPE Saúde Diário</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>@upe_depre</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>44200</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Vida Universitária / Saúde UPE</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>PE</t>
         </is>
       </c>
     </row>
@@ -25939,6 +26918,7 @@
           <t>cuiabamt300@gmail.com</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>MT</t>
@@ -25999,6 +26979,7 @@
           <t>folhamax@gmail.com</t>
         </is>
       </c>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>MT</t>
@@ -26026,6 +27007,7 @@
           <t>contato@newscuiaba.com.br</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>MT</t>
@@ -26048,6 +27030,8 @@
           <t>https://startupi.com.br/</t>
         </is>
       </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>MT</t>
@@ -26109,6 +27093,7 @@
           <t>contato@diariomatogrosso.com.br</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
           <t>MT</t>
@@ -26234,6 +27219,7 @@
           <t>aleapra@gmail.com</t>
         </is>
       </c>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>MT</t>
@@ -26448,6 +27434,8 @@
           <t>http://www.boamidia.com.br/</t>
         </is>
       </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
           <t>MT</t>
@@ -26571,6 +27559,8 @@
           <t>https://www.toquedealerta.com.br/</t>
         </is>
       </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
           <t>MT</t>
@@ -26695,6 +27685,7 @@
           <t>redacao@altnoticias.com.br</t>
         </is>
       </c>
+      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
           <t>MT</t>
@@ -26846,6 +27837,7 @@
           <t>http://www.midiarural.com.br/</t>
         </is>
       </c>
+      <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
           <t>(65) 9 99934367</t>
@@ -27066,6 +28058,7 @@
           <t>https://www.campograndenews.com.br/</t>
         </is>
       </c>
+      <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
           <t>(67) 99669-9563</t>
@@ -27221,6 +28214,7 @@
           <t>https://www.jpnews.com.br/</t>
         </is>
       </c>
+      <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
           <t>(67) 99229.0519</t>
@@ -27312,6 +28306,8 @@
           <t>http://www.primeiranoticia.ufms.br/</t>
         </is>
       </c>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
           <t>MS</t>
@@ -27751,6 +28747,8 @@
 (63) 99997- 2522</t>
         </is>
       </c>
+      <c r="C74" t="inlineStr"/>
+      <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr">
         <is>
           <t>TO</t>
@@ -27779,6 +28777,7 @@
 comercial@arnaldofilho.com.br</t>
         </is>
       </c>
+      <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr">
         <is>
           <t>TO</t>
@@ -27801,6 +28800,7 @@
           <t>https://gazetadocerrado.com.br/contato</t>
         </is>
       </c>
+      <c r="C76" t="inlineStr"/>
       <c r="D76" t="inlineStr">
         <is>
           <t>Redação:
@@ -27966,6 +28966,7 @@
  surgiu.com@hotmail.com</t>
         </is>
       </c>
+      <c r="C81" t="inlineStr"/>
       <c r="D81" t="inlineStr">
         <is>
           <t>(63) 9 9272-9920</t>
@@ -28026,6 +29027,7 @@
           <t>https://www.agenciatocantins.com.br/contato</t>
         </is>
       </c>
+      <c r="C83" t="inlineStr"/>
       <c r="D83" t="inlineStr">
         <is>
           <t>63 98500-8112</t>
@@ -28053,6 +29055,7 @@
           <t>https://araguainanoticias.com.br/anuncie</t>
         </is>
       </c>
+      <c r="C84" t="inlineStr"/>
       <c r="D84" t="inlineStr">
         <is>
           <t>(63) 9 9283-3171 
@@ -28081,6 +29084,7 @@
           <t>https://www.emaisgoias.com.br/</t>
         </is>
       </c>
+      <c r="C85" t="inlineStr"/>
       <c r="D85" t="inlineStr">
         <is>
           <t>(62) 3259-6500 / (62) 98272-3896</t>
@@ -28177,6 +29181,7 @@
           <t>altairtavares@diariodegoias.com.br</t>
         </is>
       </c>
+      <c r="D88" t="inlineStr"/>
       <c r="E88" t="inlineStr">
         <is>
           <t>GO</t>
@@ -28204,6 +29209,7 @@
           <t>redacao@folhaz.com.br / comercial@folhaz.com.br</t>
         </is>
       </c>
+      <c r="D89" t="inlineStr"/>
       <c r="E89" t="inlineStr">
         <is>
           <t>GO</t>
@@ -28450,6 +29456,7 @@
           <t>https://diariodeaparecida.com.br/</t>
         </is>
       </c>
+      <c r="C97" t="inlineStr"/>
       <c r="D97" t="inlineStr">
         <is>
           <t>(62) 3280-7894 / (62)3548-4964 / (62)99176-7917</t>
@@ -28482,6 +29489,7 @@
           <t>jornalismo1@ver7.com.br / comercial1@ver7.com.br</t>
         </is>
       </c>
+      <c r="D98" t="inlineStr"/>
       <c r="E98" t="inlineStr">
         <is>
           <t>GO</t>
@@ -28541,6 +29549,7 @@
           <t>portalnossogoiais@gmail.com</t>
         </is>
       </c>
+      <c r="D100" t="inlineStr"/>
       <c r="E100" t="inlineStr">
         <is>
           <t>GO</t>
@@ -28632,6 +29641,7 @@
           <t>danilopetmat@gmail.com / weverton@portal6.com.br / caiohenrique@portal6.com.br / matheus@portal6.com.br</t>
         </is>
       </c>
+      <c r="D103" t="inlineStr"/>
       <c r="E103" t="inlineStr">
         <is>
           <t>GO</t>
@@ -28686,6 +29696,7 @@
           <t>https://dol.com.br/</t>
         </is>
       </c>
+      <c r="C105" t="inlineStr"/>
       <c r="D105" t="inlineStr">
         <is>
           <t>91984126477</t>
@@ -28713,6 +29724,7 @@
           <t>https://agenciapara.com.br/</t>
         </is>
       </c>
+      <c r="C106" t="inlineStr"/>
       <c r="D106" t="inlineStr">
         <is>
           <t>(91) 3202-0900</t>
@@ -28745,6 +29757,7 @@
           <t>redepara@gmail.com</t>
         </is>
       </c>
+      <c r="D107" t="inlineStr"/>
       <c r="E107" t="inlineStr">
         <is>
           <t>PA</t>
@@ -28863,6 +29876,7 @@
           <t>correiodecarajas.com.br</t>
         </is>
       </c>
+      <c r="C111" t="inlineStr"/>
       <c r="D111" t="inlineStr">
         <is>
           <t>94 99212-4484 / 94 99149-1564</t>
@@ -28922,6 +29936,7 @@
           <t>pebinhadeacucar.com.br</t>
         </is>
       </c>
+      <c r="C113" t="inlineStr"/>
       <c r="D113" t="inlineStr">
         <is>
           <t>(94) 99121-9293 (whatsapp) | (94) 98134-2558</t>
@@ -28949,6 +29964,7 @@
           <t>portalgiroitb@gmail.com</t>
         </is>
       </c>
+      <c r="C114" t="inlineStr"/>
       <c r="D114" t="inlineStr">
         <is>
           <t>93 99158-7113 / 93 9140-7928 / 93 99156-8842</t>
@@ -29008,6 +30024,7 @@
           <t>zedudu.com.br</t>
         </is>
       </c>
+      <c r="C116" t="inlineStr"/>
       <c r="D116" t="inlineStr">
         <is>
           <t>94 98114 6363</t>
@@ -29131,6 +30148,7 @@
           <t>www.jesocarneiro.com.br</t>
         </is>
       </c>
+      <c r="C120" t="inlineStr"/>
       <c r="D120" t="inlineStr">
         <is>
           <t>93 99141-3040</t>
@@ -29163,6 +30181,7 @@
           <t>redepara@gmail.com</t>
         </is>
       </c>
+      <c r="D121" t="inlineStr"/>
       <c r="E121" t="inlineStr">
         <is>
           <t>PA</t>
@@ -29249,6 +30268,7 @@
           <t>oestadonet.com.br</t>
         </is>
       </c>
+      <c r="C124" t="inlineStr"/>
       <c r="D124" t="inlineStr">
         <is>
           <t>93 98414-5298</t>
@@ -29276,6 +30296,7 @@
           <t>portalcultura.com.br</t>
         </is>
       </c>
+      <c r="C125" t="inlineStr"/>
       <c r="D125" t="inlineStr">
         <is>
           <t>(91) 4005 7725</t>
@@ -29335,6 +30356,7 @@
           <t>https://d24am.com/</t>
         </is>
       </c>
+      <c r="C127" t="inlineStr"/>
       <c r="D127" t="inlineStr">
         <is>
           <t>(92) 3643-5080</t>
@@ -29875,6 +30897,7 @@
           <t>https://www.ronoticias.com.br/</t>
         </is>
       </c>
+      <c r="C144" t="inlineStr"/>
       <c r="D144" t="inlineStr">
         <is>
           <t>(69) 3322 2626</t>
@@ -29908,6 +30931,7 @@
 faleconosco@ac24horas.com</t>
         </is>
       </c>
+      <c r="D145" t="inlineStr"/>
       <c r="E145" t="inlineStr">
         <is>
           <t>AC</t>
@@ -29964,6 +30988,7 @@
           <t>https://agazeta.net/contato/</t>
         </is>
       </c>
+      <c r="C147" t="inlineStr"/>
       <c r="D147" t="inlineStr">
         <is>
           <t>(68)99989-1042</t>
@@ -29991,6 +31016,7 @@
           <t>https://www.oriobranco.net/</t>
         </is>
       </c>
+      <c r="C148" t="inlineStr"/>
       <c r="D148" t="inlineStr">
         <is>
           <t>69 999515337 
@@ -30024,6 +31050,7 @@
           <t>jornalatribunac@gmail.com</t>
         </is>
       </c>
+      <c r="D149" t="inlineStr"/>
       <c r="E149" t="inlineStr">
         <is>
           <t>AC</t>
@@ -30046,6 +31073,8 @@
           <t>https://www.instagram.com/projetoceeb/</t>
         </is>
       </c>
+      <c r="C150" t="inlineStr"/>
+      <c r="D150" t="inlineStr"/>
       <c r="E150" t="inlineStr">
         <is>
           <t>MA</t>
@@ -30068,6 +31097,8 @@
           <t>https://www.instagram.com/socialmidialarissa/</t>
         </is>
       </c>
+      <c r="C151" t="inlineStr"/>
+      <c r="D151" t="inlineStr"/>
       <c r="E151" t="inlineStr">
         <is>
           <t>SP</t>
@@ -30090,6 +31121,8 @@
           <t>https://www.instagram.com/auin_unesp/</t>
         </is>
       </c>
+      <c r="C152" t="inlineStr"/>
+      <c r="D152" t="inlineStr"/>
       <c r="E152" t="inlineStr">
         <is>
           <t>SP</t>
@@ -30112,6 +31145,8 @@
           <t>https://www.instagram.com/inovaunicamp/</t>
         </is>
       </c>
+      <c r="C153" t="inlineStr"/>
+      <c r="D153" t="inlineStr"/>
       <c r="E153" t="inlineStr">
         <is>
           <t>SP</t>
@@ -30134,6 +31169,8 @@
           <t>https://www.instagram.com/inovacao.ufscar/</t>
         </is>
       </c>
+      <c r="C154" t="inlineStr"/>
+      <c r="D154" t="inlineStr"/>
       <c r="E154" t="inlineStr">
         <is>
           <t>SP</t>
@@ -30156,6 +31193,8 @@
           <t>https://www.instagram.com/pulsehub/</t>
         </is>
       </c>
+      <c r="C155" t="inlineStr"/>
+      <c r="D155" t="inlineStr"/>
       <c r="E155" t="inlineStr">
         <is>
           <t>SP</t>
@@ -30178,6 +31217,8 @@
           <t>https://www.instagram.com/nofrontempoderamento/</t>
         </is>
       </c>
+      <c r="C156" t="inlineStr"/>
+      <c r="D156" t="inlineStr"/>
       <c r="E156" t="inlineStr">
         <is>
           <t>SP</t>
@@ -30200,6 +31241,8 @@
           <t>15997016317</t>
         </is>
       </c>
+      <c r="C157" t="inlineStr"/>
+      <c r="D157" t="inlineStr"/>
       <c r="E157" t="inlineStr">
         <is>
           <t>SP</t>
@@ -30222,6 +31265,8 @@
           <t>11970820070</t>
         </is>
       </c>
+      <c r="C158" t="inlineStr"/>
+      <c r="D158" t="inlineStr"/>
       <c r="E158" t="inlineStr">
         <is>
           <t>SP</t>
@@ -30244,6 +31289,8 @@
           <t>https://centrodemidiasp.educacao.sp.gov.br/parceiros/</t>
         </is>
       </c>
+      <c r="C159" t="inlineStr"/>
+      <c r="D159" t="inlineStr"/>
       <c r="E159" t="inlineStr">
         <is>
           <t>SP</t>
@@ -30266,6 +31313,8 @@
           <t>https://www.instagram.com/dupla.em.acao/</t>
         </is>
       </c>
+      <c r="C160" t="inlineStr"/>
+      <c r="D160" t="inlineStr"/>
       <c r="E160" t="inlineStr">
         <is>
           <t>SP</t>
@@ -30288,6 +31337,8 @@
           <t>https://instagram.com/nacomunicacao?utm_medium=copy_link</t>
         </is>
       </c>
+      <c r="C161" t="inlineStr"/>
+      <c r="D161" t="inlineStr"/>
       <c r="E161" t="inlineStr">
         <is>
           <t>SP</t>
@@ -30310,6 +31361,8 @@
           <t>https://instagram.com/agenciajhma?utm_medium=copy_link</t>
         </is>
       </c>
+      <c r="C162" t="inlineStr"/>
+      <c r="D162" t="inlineStr"/>
       <c r="E162" t="inlineStr">
         <is>
           <t>SP</t>
@@ -30332,6 +31385,8 @@
           <t>https://instagram.com/conectecomunicacao?utm_medium=copy_link</t>
         </is>
       </c>
+      <c r="C163" t="inlineStr"/>
+      <c r="D163" t="inlineStr"/>
       <c r="E163" t="inlineStr">
         <is>
           <t>SP</t>
@@ -30354,6 +31409,8 @@
           <t>https://instagram.com/agenciavision?utm_medium=copy_link</t>
         </is>
       </c>
+      <c r="C164" t="inlineStr"/>
+      <c r="D164" t="inlineStr"/>
       <c r="E164" t="inlineStr">
         <is>
           <t>SP</t>
@@ -30376,6 +31433,8 @@
           <t>https://instagram.com/agenciamangata?utm_medium=copy_link</t>
         </is>
       </c>
+      <c r="C165" t="inlineStr"/>
+      <c r="D165" t="inlineStr"/>
       <c r="E165" t="inlineStr">
         <is>
           <t>SP</t>
@@ -30398,6 +31457,8 @@
           <t>https://instagram.com/agenciaigloo?utm_medium=copy_link</t>
         </is>
       </c>
+      <c r="C166" t="inlineStr"/>
+      <c r="D166" t="inlineStr"/>
       <c r="E166" t="inlineStr">
         <is>
           <t>SP</t>
@@ -30420,6 +31481,8 @@
           <t>https://instagram.com/theleadag?utm_medium=copy_link</t>
         </is>
       </c>
+      <c r="C167" t="inlineStr"/>
+      <c r="D167" t="inlineStr"/>
       <c r="E167" t="inlineStr">
         <is>
           <t>SP</t>
@@ -30442,6 +31505,8 @@
           <t>https://www.instagram.com/vaidebolsa_/</t>
         </is>
       </c>
+      <c r="C168" t="inlineStr"/>
+      <c r="D168" t="inlineStr"/>
       <c r="E168" t="inlineStr">
         <is>
           <t>RJ</t>
@@ -30464,6 +31529,8 @@
           <t>https://www.instagram.com/oficialacademicos/</t>
         </is>
       </c>
+      <c r="C169" t="inlineStr"/>
+      <c r="D169" t="inlineStr"/>
       <c r="E169" t="inlineStr">
         <is>
           <t>RJ</t>
@@ -30486,6 +31553,8 @@
           <t>https://www.instagram.com/1mioportunidades/</t>
         </is>
       </c>
+      <c r="C170" t="inlineStr"/>
+      <c r="D170" t="inlineStr"/>
       <c r="E170" t="inlineStr">
         <is>
           <t>RJ</t>
@@ -30508,6 +31577,8 @@
           <t>https://www.instagram.com/inoc_b/</t>
         </is>
       </c>
+      <c r="C171" t="inlineStr"/>
+      <c r="D171" t="inlineStr"/>
       <c r="E171" t="inlineStr">
         <is>
           <t>RJ</t>
@@ -30530,6 +31601,8 @@
           <t>https://instagram.com/agenciawinkmidia?utm_medium=copy_link</t>
         </is>
       </c>
+      <c r="C172" t="inlineStr"/>
+      <c r="D172" t="inlineStr"/>
       <c r="E172" t="inlineStr">
         <is>
           <t>RJ</t>
@@ -30552,6 +31625,8 @@
           <t>https://instagram.com/agenciaguppy?utm_medium=copy_link</t>
         </is>
       </c>
+      <c r="C173" t="inlineStr"/>
+      <c r="D173" t="inlineStr"/>
       <c r="E173" t="inlineStr">
         <is>
           <t>RJ</t>
@@ -30574,6 +31649,8 @@
           <t>https://instagram.com/agenciam2br?utm_medium=copy_link</t>
         </is>
       </c>
+      <c r="C174" t="inlineStr"/>
+      <c r="D174" t="inlineStr"/>
       <c r="E174" t="inlineStr">
         <is>
           <t>RJ</t>
@@ -30596,6 +31673,8 @@
           <t>https://instagram.com/agestrategica?utm_medium=copy_link</t>
         </is>
       </c>
+      <c r="C175" t="inlineStr"/>
+      <c r="D175" t="inlineStr"/>
       <c r="E175" t="inlineStr">
         <is>
           <t>RJ</t>
@@ -30618,6 +31697,8 @@
           <t>https://instagram.com/donacomunicacao?utm_medium=copy_link</t>
         </is>
       </c>
+      <c r="C176" t="inlineStr"/>
+      <c r="D176" t="inlineStr"/>
       <c r="E176" t="inlineStr">
         <is>
           <t>RJ</t>
@@ -30640,6 +31721,8 @@
           <t>https://www.instagram.com/lin_itba/</t>
         </is>
       </c>
+      <c r="C177" t="inlineStr"/>
+      <c r="D177" t="inlineStr"/>
       <c r="E177" t="inlineStr">
         <is>
           <t>MG</t>
@@ -30662,6 +31745,8 @@
           <t>https://instagram.com/agencia_ecos?utm_medium=copy_link.</t>
         </is>
       </c>
+      <c r="C178" t="inlineStr"/>
+      <c r="D178" t="inlineStr"/>
       <c r="E178" t="inlineStr">
         <is>
           <t>MG</t>
@@ -30684,6 +31769,8 @@
           <t>https://instagram.com/thetpropaganda?utm_medium=copy_link</t>
         </is>
       </c>
+      <c r="C179" t="inlineStr"/>
+      <c r="D179" t="inlineStr"/>
       <c r="E179" t="inlineStr">
         <is>
           <t>MG</t>
@@ -30706,6 +31793,8 @@
           <t>https://instagram.com/agencia_lmbrt?utm_medium=copy_link</t>
         </is>
       </c>
+      <c r="C180" t="inlineStr"/>
+      <c r="D180" t="inlineStr"/>
       <c r="E180" t="inlineStr">
         <is>
           <t>MG</t>
@@ -30728,6 +31817,8 @@
           <t>https://instagram.com/mddigital_agencia?utm_medium=copy_link</t>
         </is>
       </c>
+      <c r="C181" t="inlineStr"/>
+      <c r="D181" t="inlineStr"/>
       <c r="E181" t="inlineStr">
         <is>
           <t>MG</t>
@@ -30750,6 +31841,8 @@
           <t>(31)3879-8007</t>
         </is>
       </c>
+      <c r="C182" t="inlineStr"/>
+      <c r="D182" t="inlineStr"/>
       <c r="E182" t="inlineStr">
         <is>
           <t>MG</t>
@@ -30772,6 +31865,8 @@
           <t>(34)3312-4414</t>
         </is>
       </c>
+      <c r="C183" t="inlineStr"/>
+      <c r="D183" t="inlineStr"/>
       <c r="E183" t="inlineStr">
         <is>
           <t>MG</t>
@@ -30794,6 +31889,8 @@
           <t>(31)3335-0854</t>
         </is>
       </c>
+      <c r="C184" t="inlineStr"/>
+      <c r="D184" t="inlineStr"/>
       <c r="E184" t="inlineStr">
         <is>
           <t>MG</t>
@@ -30816,6 +31913,8 @@
           <t>(31)99665-7799</t>
         </is>
       </c>
+      <c r="C185" t="inlineStr"/>
+      <c r="D185" t="inlineStr"/>
       <c r="E185" t="inlineStr">
         <is>
           <t>MG</t>
@@ -30838,6 +31937,8 @@
           <t>(31)987953506</t>
         </is>
       </c>
+      <c r="C186" t="inlineStr"/>
+      <c r="D186" t="inlineStr"/>
       <c r="E186" t="inlineStr">
         <is>
           <t>MG</t>
@@ -30860,6 +31961,8 @@
           <t>https://instagram.com/boa_imagem?utm_medium=copy_link</t>
         </is>
       </c>
+      <c r="C187" t="inlineStr"/>
+      <c r="D187" t="inlineStr"/>
       <c r="E187" t="inlineStr">
         <is>
           <t>DF</t>
@@ -30882,6 +31985,8 @@
           <t>https://instagram.com/agencialesspaper001?utm_medium=copy_link</t>
         </is>
       </c>
+      <c r="C188" t="inlineStr"/>
+      <c r="D188" t="inlineStr"/>
       <c r="E188" t="inlineStr">
         <is>
           <t>DF</t>
@@ -30904,6 +32009,8 @@
           <t>(61)98201-0600</t>
         </is>
       </c>
+      <c r="C189" t="inlineStr"/>
+      <c r="D189" t="inlineStr"/>
       <c r="E189" t="inlineStr">
         <is>
           <t>DF</t>
@@ -30926,6 +32033,8 @@
           <t>(61)3443-5450</t>
         </is>
       </c>
+      <c r="C190" t="inlineStr"/>
+      <c r="D190" t="inlineStr"/>
       <c r="E190" t="inlineStr">
         <is>
           <t>DF</t>
@@ -30948,6 +32057,8 @@
           <t>(61)3032-8811</t>
         </is>
       </c>
+      <c r="C191" t="inlineStr"/>
+      <c r="D191" t="inlineStr"/>
       <c r="E191" t="inlineStr">
         <is>
           <t>DF</t>
@@ -30970,6 +32081,8 @@
           <t>(61)99169-5678</t>
         </is>
       </c>
+      <c r="C192" t="inlineStr"/>
+      <c r="D192" t="inlineStr"/>
       <c r="E192" t="inlineStr">
         <is>
           <t>DF</t>
@@ -30992,6 +32105,8 @@
           <t>(61)3964-0963</t>
         </is>
       </c>
+      <c r="C193" t="inlineStr"/>
+      <c r="D193" t="inlineStr"/>
       <c r="E193" t="inlineStr">
         <is>
           <t>DF</t>
@@ -31014,6 +32129,8 @@
           <t>(61)4103-6558</t>
         </is>
       </c>
+      <c r="C194" t="inlineStr"/>
+      <c r="D194" t="inlineStr"/>
       <c r="E194" t="inlineStr">
         <is>
           <t>DF</t>
@@ -31036,6 +32153,8 @@
           <t>(61)3297-5436</t>
         </is>
       </c>
+      <c r="C195" t="inlineStr"/>
+      <c r="D195" t="inlineStr"/>
       <c r="E195" t="inlineStr">
         <is>
           <t>DF</t>
@@ -31099,10 +32218,10 @@
           <t>Núcleo Bauru</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>15997016317</t>
-        </is>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="n">
+        <v>15997016317</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -31121,10 +32240,10 @@
           <t>Brasil Jr</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>11970820070</t>
-        </is>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="n">
+        <v>11970820070</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -31143,10 +32262,10 @@
           <t>CA Eng. Quimíca UFMT | Enactus UFMT</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>6593616791</t>
-        </is>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="n">
+        <v>6593616791</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -31165,10 +32284,10 @@
           <t>Instituto Four</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>3388546292</t>
-        </is>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="n">
+        <v>3388546292</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -31192,6 +32311,8 @@
           <t>https://www.instagram.com/_startcoding/</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31214,6 +32335,8 @@
           <t>https://www.instagram.com/1mioportunidades/</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31236,6 +32359,8 @@
           <t>https://www.instagram.com/4pluslanguage/</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31258,6 +32383,8 @@
           <t>https://www.instagram.com/abglt.oficial/</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31280,6 +32407,8 @@
           <t>https://www.instagram.com/abrapsoficial/</t>
         </is>
       </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31302,6 +32431,8 @@
           <t>https://www.instagram.com/abrindoportas_ong/</t>
         </is>
       </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31324,6 +32455,8 @@
           <t>https://www.instagram.com/academialinguistica/</t>
         </is>
       </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31346,6 +32479,8 @@
           <t>https://www.instagram.com/oficialacademicos/</t>
         </is>
       </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31368,6 +32503,8 @@
           <t>https://www.instagram.com/acientistadedados/</t>
         </is>
       </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31390,6 +32527,8 @@
           <t>https://www.instagram.com/actumbrazil/</t>
         </is>
       </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31412,6 +32551,8 @@
           <t>https://www.instagram.com/adriana.saty/</t>
         </is>
       </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31434,6 +32575,8 @@
           <t>https://www.instagram.com/transformacaoofc/</t>
         </is>
       </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31456,6 +32599,8 @@
           <t>https://www.instagram.com/afrontlab/</t>
         </is>
       </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31478,6 +32623,8 @@
           <t>https://www.instagram.com/inovacao.ufscar/</t>
         </is>
       </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31500,6 +32647,8 @@
           <t>https://www.instagram.com/inovaunicamp/</t>
         </is>
       </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31522,6 +32671,8 @@
           <t>https://www.instagram.com/auin_unesp/</t>
         </is>
       </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31544,6 +32695,8 @@
           <t>https://www.instagram.com/ago.social/</t>
         </is>
       </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31566,6 +32719,8 @@
           <t>https://www.instagram.com/aiesecnobrasil/</t>
         </is>
       </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31588,6 +32743,8 @@
           <t>https://www.instagram.com/akasulo/</t>
         </is>
       </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31610,6 +32767,8 @@
           <t>https://www.instagram.com/akitaonrails/</t>
         </is>
       </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31632,6 +32791,8 @@
           <t>https://www.instagram.com/aldeiadofuturo/</t>
         </is>
       </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31654,6 +32815,8 @@
           <t>https://www.instagram.com/alumna_br/</t>
         </is>
       </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31676,6 +32839,8 @@
           <t>https://www.instagram.com/alunoaocubo/</t>
         </is>
       </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31698,6 +32863,8 @@
           <t>https://www.instagram.com/alunosporalunos/</t>
         </is>
       </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31720,6 +32887,8 @@
           <t>https://www.instagram.com/anapaula.sql/</t>
         </is>
       </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31742,6 +32911,8 @@
           <t>https://www.instagram.com/andadireito/</t>
         </is>
       </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31764,6 +32935,8 @@
           <t>https://www.instagram.com/carinhadoti/</t>
         </is>
       </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31786,6 +32959,8 @@
           <t>https://www.instagram.com/aplicaeasy/</t>
         </is>
       </c>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31808,6 +32983,8 @@
           <t>https://www.instagram.com/ashokabrasil/</t>
         </is>
       </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31830,6 +33007,8 @@
           <t>https://www.instagram.com/odarasocial/</t>
         </is>
       </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31852,6 +33031,8 @@
           <t>https://www.instagram.com/associacao.falamulher/</t>
         </is>
       </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31874,6 +33055,8 @@
           <t>https://www.instagram.com/atados/</t>
         </is>
       </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31896,6 +33079,8 @@
           <t>https://www.instagram.com/aaamercurio/</t>
         </is>
       </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31918,6 +33103,8 @@
           <t>https://www.instagram.com/attekitadev/</t>
         </is>
       </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31940,6 +33127,8 @@
           <t>https://www.instagram.com/automatizeigeral/</t>
         </is>
       </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31962,6 +33151,8 @@
           <t>https://www.instagram.com/autoticbrasil/</t>
         </is>
       </c>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
           <t>BR</t>
@@ -31984,6 +33175,8 @@
           <t>https://www.instagram.com/binamidia/</t>
         </is>
       </c>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32006,6 +33199,8 @@
           <t>https://www.instagram.com/biotec_op/</t>
         </is>
       </c>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32028,6 +33223,8 @@
           <t>https://www.instagram.com/biudmarketing/</t>
         </is>
       </c>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32050,6 +33247,8 @@
           <t>https://www.instagram.com/projetobraie/</t>
         </is>
       </c>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32072,6 +33271,8 @@
           <t>https://www.instagram.com/brain.innovation/</t>
         </is>
       </c>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32094,6 +33295,8 @@
           <t>https://www.instagram.com/gobrasa/</t>
         </is>
       </c>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32116,6 +33319,8 @@
           <t>https://www.instagram.com/bjnoinsta/</t>
         </is>
       </c>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32138,6 +33343,8 @@
           <t>https://www.instagram.com/brasilcode_/</t>
         </is>
       </c>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32160,6 +33367,8 @@
           <t>https://www.instagram.com/brazil_conference/</t>
         </is>
       </c>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32182,6 +33391,8 @@
           <t>https://www.instagram.com/braziliansintech/</t>
         </is>
       </c>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32204,6 +33415,8 @@
           <t>https://www.instagram.com/cafeparaprogramar/</t>
         </is>
       </c>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32226,6 +33439,8 @@
           <t>https://www.instagram.com/caiommoreno/</t>
         </is>
       </c>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32248,6 +33463,8 @@
           <t>https://www.instagram.com/canalnovomundo/</t>
         </is>
       </c>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32270,6 +33487,8 @@
           <t>https://www.instagram.com/capibagirls/</t>
         </is>
       </c>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32292,6 +33511,8 @@
           <t>https://www.instagram.com/carlos_melo.py/</t>
         </is>
       </c>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32314,6 +33535,8 @@
           <t>https://www.instagram.com/centrodaautomacao4.0/</t>
         </is>
       </c>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32336,6 +33559,8 @@
           <t>https://www.instagram.com/centrodetecnologia_ufpi/</t>
         </is>
       </c>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32358,6 +33583,8 @@
           <t>https://www.instagram.com/cervejacomcodigo.com.br/</t>
         </is>
       </c>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32380,6 +33607,8 @@
           <t>https://www.instagram.com/chatclass_brasil/</t>
         </is>
       </c>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32402,6 +33631,8 @@
           <t>https://www.instagram.com/cicloliterario/</t>
         </is>
       </c>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32424,6 +33655,8 @@
           <t>https://www.instagram.com/cidadaopromundo/</t>
         </is>
       </c>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32446,6 +33679,8 @@
           <t>https://www.instagram.com/cienciaeelas/</t>
         </is>
       </c>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32468,6 +33703,8 @@
           <t>https://www.instagram.com/cienciadedadosbrasil/</t>
         </is>
       </c>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32490,6 +33727,8 @@
           <t>https://www.instagram.com/cienciaeelas//</t>
         </is>
       </c>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32512,6 +33751,8 @@
           <t>https://www.instagram.com/cientistacriativa/</t>
         </is>
       </c>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32534,6 +33775,8 @@
           <t>https://www.instagram.com/clubeopinternacionais/</t>
         </is>
       </c>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32556,6 +33799,8 @@
           <t>https://www.instagram.com/cneg_oficial/</t>
         </is>
       </c>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32578,6 +33823,8 @@
           <t>https://www.instagram.com/coliga.digital/</t>
         </is>
       </c>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32600,6 +33847,8 @@
           <t>https://www.instagram.com/cod.agirl/</t>
         </is>
       </c>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr"/>
       <c r="E70" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32622,6 +33871,8 @@
           <t>https://www.instagram.com/codandoclub/</t>
         </is>
       </c>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32644,6 +33895,8 @@
           <t>https://www.instagram.com/codelab.ong/</t>
         </is>
       </c>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32666,6 +33919,8 @@
           <t>https://www.instagram.com/codemigas/</t>
         </is>
       </c>
+      <c r="C73" t="inlineStr"/>
+      <c r="D73" t="inlineStr"/>
       <c r="E73" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32688,6 +33943,8 @@
           <t>https://www.instagram.com/cojovem.br/</t>
         </is>
       </c>
+      <c r="C74" t="inlineStr"/>
+      <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32710,6 +33967,8 @@
           <t>https://www.instagram.com/cojuv_piaui/</t>
         </is>
       </c>
+      <c r="C75" t="inlineStr"/>
+      <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32732,6 +33991,8 @@
           <t>https://www.instagram.com/cojuvdhpicos/</t>
         </is>
       </c>
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32754,6 +34015,8 @@
           <t>https://www.instagram.com/coletivanet/</t>
         </is>
       </c>
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="inlineStr"/>
       <c r="E77" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32776,6 +34039,8 @@
           <t>https://www.instagram.com/coletivomaracanau/</t>
         </is>
       </c>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32798,6 +34063,8 @@
           <t>https://www.instagram.com/piracemacoletivo/</t>
         </is>
       </c>
+      <c r="C79" t="inlineStr"/>
+      <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32820,6 +34087,8 @@
           <t>https://www.instagram.com/coletivoadinkrars/</t>
         </is>
       </c>
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32842,6 +34111,8 @@
           <t>https://www.instagram.com/coletivofotada/</t>
         </is>
       </c>
+      <c r="C81" t="inlineStr"/>
+      <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32864,6 +34135,8 @@
           <t>https://www.instagram.com/com.dados/</t>
         </is>
       </c>
+      <c r="C82" t="inlineStr"/>
+      <c r="D82" t="inlineStr"/>
       <c r="E82" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32886,6 +34159,8 @@
           <t>https://www.instagram.com/comodonerd/</t>
         </is>
       </c>
+      <c r="C83" t="inlineStr"/>
+      <c r="D83" t="inlineStr"/>
       <c r="E83" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32908,6 +34183,8 @@
           <t>https://www.instagram.com/compartilhe.sorrisos/</t>
         </is>
       </c>
+      <c r="C84" t="inlineStr"/>
+      <c r="D84" t="inlineStr"/>
       <c r="E84" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32930,6 +34207,8 @@
           <t>https://www.instagram.com/cje.oficial/</t>
         </is>
       </c>
+      <c r="C85" t="inlineStr"/>
+      <c r="D85" t="inlineStr"/>
       <c r="E85" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32952,6 +34231,8 @@
           <t>https://www.instagram.com/concentrodf/</t>
         </is>
       </c>
+      <c r="C86" t="inlineStr"/>
+      <c r="D86" t="inlineStr"/>
       <c r="E86" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32974,6 +34255,8 @@
           <t>https://www.instagram.com/conecta_elas/</t>
         </is>
       </c>
+      <c r="C87" t="inlineStr"/>
+      <c r="D87" t="inlineStr"/>
       <c r="E87" t="inlineStr">
         <is>
           <t>BR</t>
@@ -32996,6 +34279,8 @@
           <t>https://www.instagram.com/coeducabrasil/</t>
         </is>
       </c>
+      <c r="C88" t="inlineStr"/>
+      <c r="D88" t="inlineStr"/>
       <c r="E88" t="inlineStr">
         <is>
           <t>BR</t>
@@ -33018,6 +34303,8 @@
           <t>https://www.instagram.com/conexaosocial/</t>
         </is>
       </c>
+      <c r="C89" t="inlineStr"/>
+      <c r="D89" t="inlineStr"/>
       <c r="E89" t="inlineStr">
         <is>
           <t>BR</t>
@@ -33040,6 +34327,8 @@
           <t>https://www.instagram.com/conjuvebr/</t>
         </is>
       </c>
+      <c r="C90" t="inlineStr"/>
+      <c r="D90" t="inlineStr"/>
       <c r="E90" t="inlineStr">
         <is>
           <t>BR</t>
@@ -33062,6 +34351,8 @@
           <t>https://www.instagram.com/conselhopsicologiars/</t>
         </is>
       </c>
+      <c r="C91" t="inlineStr"/>
+      <c r="D91" t="inlineStr"/>
       <c r="E91" t="inlineStr">
         <is>
           <t>BR</t>
@@ -33084,6 +34375,8 @@
           <t>https://www.instagram.com/construindofuturobr/</t>
         </is>
       </c>
+      <c r="C92" t="inlineStr"/>
+      <c r="D92" t="inlineStr"/>
       <c r="E92" t="inlineStr">
         <is>
           <t>BR</t>
@@ -33106,6 +34399,8 @@
           <t>https://www.instagram.com/cosmicas.tomieohtake/</t>
         </is>
       </c>
+      <c r="C93" t="inlineStr"/>
+      <c r="D93" t="inlineStr"/>
       <c r="E93" t="inlineStr">
         <is>
           <t>BR</t>
@@ -33128,6 +34423,8 @@
           <t>https://www.instagram.com/crcjovempi/</t>
         </is>
       </c>
+      <c r="C94" t="inlineStr"/>
+      <c r="D94" t="inlineStr"/>
       <c r="E94" t="inlineStr">
         <is>
           <t>BR</t>
@@ -33150,6 +34447,8 @@
           <t>https://www.instagram.com/create.se/</t>
         </is>
       </c>
+      <c r="C95" t="inlineStr"/>
+      <c r="D95" t="inlineStr"/>
       <c r="E95" t="inlineStr">
         <is>
           <t>BR</t>
@@ -33172,6 +34471,8 @@
           <t>https://www.instagram.com/cjr.unb/</t>
         </is>
       </c>
+      <c r="C96" t="inlineStr"/>
+      <c r="D96" t="inlineStr"/>
       <c r="E96" t="inlineStr">
         <is>
           <t>BR</t>
@@ -33194,6 +34495,8 @@
           <t>https://www.instagram.com/cubos.io/</t>
         </is>
       </c>
+      <c r="C97" t="inlineStr"/>
+      <c r="D97" t="inlineStr"/>
       <c r="E97" t="inlineStr">
         <is>
           <t>BR</t>
@@ -33216,6 +34519,8 @@
           <t>https://www.instagram.com/culturadev_/</t>
         </is>
       </c>
+      <c r="C98" t="inlineStr"/>
+      <c r="D98" t="inlineStr"/>
       <c r="E98" t="inlineStr">
         <is>
           <t>BR</t>
@@ -33238,6 +34543,8 @@
           <t>https://www.instagram.com/cursinhofeausp/</t>
         </is>
       </c>
+      <c r="C99" t="inlineStr"/>
+      <c r="D99" t="inlineStr"/>
       <c r="E99" t="inlineStr">
         <is>
           <t>BR</t>
@@ -33260,6 +34567,8 @@
           <t>https://www.instagram.com/cursinhopoliusp/</t>
         </is>
       </c>
+      <c r="C100" t="inlineStr"/>
+      <c r="D100" t="inlineStr"/>
       <c r="E100" t="inlineStr">
         <is>
           <t>BR</t>
@@ -33282,6 +34591,8 @@
           <t>https://www.instagram.com/cursinho.insper/</t>
         </is>
       </c>
+      <c r="C101" t="inlineStr"/>
+      <c r="D101" t="inlineStr"/>
       <c r="E101" t="inlineStr">
         <is>
           <t>BR</t>
@@ -33304,6 +34615,8 @@
           <t>https://www.instagram.com/cursoipe/</t>
         </is>
       </c>
+      <c r="C102" t="inlineStr"/>
+      <c r="D102" t="inlineStr"/>
       <c r="E102" t="inlineStr">
         <is>
           <t>BR</t>
@@ -33326,6 +34639,8 @@
           <t>https://www.instagram.com/daltro.projeto/</t>
         </is>
       </c>
+      <c r="C103" t="inlineStr"/>
+      <c r="D103" t="inlineStr"/>
       <c r="E103" t="inlineStr">
         <is>
           <t>BR</t>
@@ -33348,6 +34663,8 @@
           <t>https://www.instagram.com/dados.karen/</t>
         </is>
       </c>
+      <c r="C104" t="inlineStr"/>
+      <c r="D104" t="inlineStr"/>
       <c r="E104" t="inlineStr">
         <is>
           <t>BR</t>
@@ -33370,6 +34687,8 @@
           <t>https://www.instagram.com/danielematos_rhlovers/</t>
         </is>
       </c>
+      <c r="C105" t="inlineStr"/>
+      <c r="D105" t="inlineStr"/>
       <c r="E105" t="inlineStr">
         <is>
           <t>BR</t>

</xml_diff>